<commit_message>
Update NBA features + predictions: 2026-10-03 22:51
</commit_message>
<xml_diff>
--- a/nba-backend/data_delivery/nba_feature_workbook_20261003.xlsx
+++ b/nba-backend/data_delivery/nba_feature_workbook_20261003.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nba-prod-v2.5-epm</t>
+          <t>nba-prod-v2.6-rapm</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Point-in-time exclusion from the projected lineup pool for the pl_epm_* family (Out/Doubtful/Recovery removed from that game only).</t>
+          <t>Point-in-time exclusion from the projected lineup pool for the pl_rapm_* family (Out/Doubtful/Recovery removed from that game only).</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -5835,17 +5835,17 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_away</t>
+          <t>pl_rapm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -5867,17 +5867,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_home</t>
+          <t>pl_rapm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -5899,17 +5899,17 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_diff</t>
+          <t>pl_rapm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -5931,17 +5931,17 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_away</t>
+          <t>pl_rapm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -5963,17 +5963,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_home</t>
+          <t>pl_rapm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -5995,17 +5995,17 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_diff</t>
+          <t>pl_rapm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -6027,17 +6027,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_away</t>
+          <t>pl_rapm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -6059,17 +6059,17 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_home</t>
+          <t>pl_rapm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -6091,17 +6091,17 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_diff</t>
+          <t>pl_rapm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -8309,7 +8309,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_away</t>
+          <t>pl_rapm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="b">
@@ -8322,7 +8322,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_home</t>
+          <t>pl_rapm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="b">
@@ -8335,7 +8335,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_diff</t>
+          <t>pl_rapm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="b">
@@ -8348,7 +8348,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_away</t>
+          <t>pl_rapm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="b">
@@ -8361,7 +8361,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_home</t>
+          <t>pl_rapm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="b">
@@ -8374,7 +8374,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_diff</t>
+          <t>pl_rapm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="b">
@@ -8387,7 +8387,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_away</t>
+          <t>pl_rapm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="b">
@@ -8400,7 +8400,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_home</t>
+          <t>pl_rapm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="b">
@@ -8413,7 +8413,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_diff</t>
+          <t>pl_rapm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="b">
@@ -9020,7 +9020,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>nba-prod-v2.5-epm</t>
+          <t>nba-prod-v2.6-rapm</t>
         </is>
       </c>
     </row>
@@ -12221,7 +12221,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_away</t>
+          <t>pl_rapm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -12246,25 +12246,29 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>0.197</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_home</t>
+          <t>pl_rapm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -12289,25 +12293,29 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>0.5252</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_diff</t>
+          <t>pl_rapm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -12332,25 +12340,29 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>0.3653</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_away</t>
+          <t>pl_rapm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -12375,25 +12387,29 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>0.1977</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_home</t>
+          <t>pl_rapm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -12418,25 +12434,29 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I68" s="2" t="n">
-        <v>0.2185</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_diff</t>
+          <t>pl_rapm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -12461,25 +12481,29 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I69" s="2" t="n">
-        <v>3.003</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_away</t>
+          <t>pl_rapm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -12504,25 +12528,29 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I70" s="2" t="n">
-        <v>0.5465</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_home</t>
+          <t>pl_rapm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -12547,25 +12575,29 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I71" s="2" t="n">
-        <v>0.111</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_diff</t>
+          <t>pl_rapm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -12590,19 +12622,23 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I72" s="2" t="n">
-        <v>1.7803</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -17321,7 +17357,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_away</t>
+          <t>pl_rapm_c_away</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -17346,25 +17382,29 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>0.197</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_home</t>
+          <t>pl_rapm_c_home</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -17389,25 +17429,29 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I65" s="2" t="n">
-        <v>0.5252</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_c_diff</t>
+          <t>pl_rapm_c_diff</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -17432,25 +17476,29 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>0.3653</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_away</t>
+          <t>pl_rapm_f_away</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -17475,25 +17523,29 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>0.1977</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_home</t>
+          <t>pl_rapm_f_home</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -17518,25 +17570,29 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I68" s="2" t="n">
-        <v>0.2185</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_f_diff</t>
+          <t>pl_rapm_f_diff</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -17561,25 +17617,29 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I69" s="2" t="n">
-        <v>3.003</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_away</t>
+          <t>pl_rapm_g_away</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -17604,25 +17664,29 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, away side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, away side</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I70" s="2" t="n">
-        <v>0.5465</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (away side)</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_home</t>
+          <t>pl_rapm_g_home</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -17647,25 +17711,29 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>position-segmented shrunk estimated plus-minus of the projected lineup, home side</t>
+          <t>position-segmented shrunk RAPM (points per game) of the projected lineup, home side</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I71" s="2" t="n">
-        <v>0.111</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive)) (home side)</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>pl_epm_g_diff</t>
+          <t>pl_rapm_g_diff</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -17690,19 +17758,23 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>home minus away gap in the position-segmented shrunk estimated plus-minus of the projected lineup</t>
+          <t>home minus away gap in the position-segmented shrunk RAPM (points per game) of the projected lineup</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk EPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I72" s="2" t="n">
-        <v>1.7803</v>
+          <t>stats.nba.com LeagueGameLog player lines -&gt; position-segmented shrunk RAPM -&gt; projected lineup average (official NBA injury report (published designations archive))</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>